<commit_message>
Update redaction timing workbooks
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F654748-8BDE-4DCF-B8EA-0C65F856E93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C226021E-B957-4E4D-9622-51CA8B3446C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="202">
   <si>
     <t>date</t>
   </si>
@@ -600,12 +611,6 @@
     <t>dead time</t>
   </si>
   <si>
-    <t>??</t>
-  </si>
-  <si>
-    <t>not a case</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 07:01:03</t>
   </si>
   <si>
@@ -631,6 +636,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>note a case</t>
+  </si>
+  <si>
+    <t>לא לחתוך</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1248,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:7">
       <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1260,7 +1271,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:7">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
@@ -1271,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:7">
       <c r="A19" s="2" t="s">
         <v>30</v>
       </c>
@@ -1282,7 +1293,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -1296,7 +1307,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
@@ -1307,7 +1318,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:7">
       <c r="A22" s="2" t="s">
         <v>33</v>
       </c>
@@ -1315,7 +1326,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:7">
       <c r="A23" s="2" t="s">
         <v>34</v>
       </c>
@@ -1326,7 +1337,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:7">
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
@@ -1337,7 +1348,7 @@
         <v>4.7546296296296295E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:7">
       <c r="A25" s="2" t="s">
         <v>36</v>
       </c>
@@ -1347,17 +1358,9 @@
       <c r="E25" s="3">
         <v>1.8576388888888889E-2</v>
       </c>
-      <c r="F25" s="3">
-        <v>3.1805555555555552E-2</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H25" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="2" t="s">
         <v>37</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>7.3530092592592591E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:7">
       <c r="A27" s="2" t="s">
         <v>38</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:7">
       <c r="A28" s="2" t="s">
         <v>39</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>0.12725694444444444</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:7">
       <c r="A29" s="2" t="s">
         <v>40</v>
       </c>
@@ -1401,7 +1404,7 @@
         <v>0.25537037037037036</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:7">
       <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
@@ -1412,7 +1415,7 @@
         <v>5.8252314814814812E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:7">
       <c r="A31" s="2" t="s">
         <v>42</v>
       </c>
@@ -1423,7 +1426,7 @@
         <v>8.5289351851851852E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:7">
       <c r="A32" s="2" t="s">
         <v>43</v>
       </c>
@@ -1434,7 +1437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:8">
       <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
@@ -1445,7 +1448,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:8">
       <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
@@ -1456,7 +1459,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
         <v>46</v>
       </c>
@@ -1467,7 +1470,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:8">
       <c r="A36" s="2" t="s">
         <v>47</v>
       </c>
@@ -1478,7 +1481,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
         <v>48</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:8">
       <c r="A38" s="2" t="s">
         <v>49</v>
       </c>
@@ -1500,7 +1503,7 @@
         <v>7.6284722222222226E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:8">
       <c r="A39" s="2" t="s">
         <v>50</v>
       </c>
@@ -1510,11 +1513,11 @@
       <c r="C39" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="H39" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
@@ -1534,10 +1537,10 @@
         <v>0.22163194444444445</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="2" t="s">
         <v>52</v>
       </c>
@@ -1548,7 +1551,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:8">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1559,7 +1562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:8">
       <c r="A43" s="2" t="s">
         <v>54</v>
       </c>
@@ -1570,7 +1573,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:8">
       <c r="A44" s="2" t="s">
         <v>55</v>
       </c>
@@ -1578,7 +1581,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:8">
       <c r="A45" s="2" t="s">
         <v>56</v>
       </c>
@@ -1589,7 +1592,7 @@
         <v>0.18371527777777777</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:8">
       <c r="A46" s="2" t="s">
         <v>57</v>
       </c>
@@ -1600,7 +1603,7 @@
         <v>0.12155092592592592</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:8">
       <c r="A47" s="2" t="s">
         <v>58</v>
       </c>
@@ -1611,7 +1614,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:8">
       <c r="A48" s="2" t="s">
         <v>59</v>
       </c>
@@ -1683,7 +1686,7 @@
         <v>0.19527777777777777</v>
       </c>
       <c r="H53" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -1702,7 +1705,7 @@
         <v>66</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C55" s="3">
         <v>9.6782407407407414E-2</v>
@@ -2029,12 +2032,8 @@
       <c r="C84" s="3">
         <v>0.12923611111111111</v>
       </c>
-      <c r="D84" s="3">
-        <v>0.15792824074074074</v>
-      </c>
-      <c r="E84" s="3">
-        <v>0.21453703703703703</v>
-      </c>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
       <c r="H84" t="s">
         <v>11</v>
       </c>
@@ -2082,11 +2081,8 @@
       <c r="C88" s="3">
         <v>5.6423611111111112E-2</v>
       </c>
-      <c r="D88" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="H88" t="s">
-        <v>11</v>
+      <c r="H88" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -2500,7 +2496,7 @@
         <v>129</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -2530,7 +2526,7 @@
         <v>132</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -2574,7 +2570,7 @@
         <v>9</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D125" s="3">
         <v>8.1180555555555561E-2</v>
@@ -2741,7 +2737,7 @@
         <v>9</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -2766,7 +2762,7 @@
         <v>151</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -2919,7 +2915,7 @@
         <v>166</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -2962,10 +2958,10 @@
         <v>171</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7">
       <c r="A161" s="2" t="s">
         <v>172</v>
       </c>
@@ -2976,7 +2972,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8">
+    <row r="162" spans="1:7">
       <c r="A162" s="2" t="s">
         <v>173</v>
       </c>
@@ -2984,7 +2980,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="163" spans="1:8">
+    <row r="163" spans="1:7">
       <c r="A163" s="2" t="s">
         <v>174</v>
       </c>
@@ -2995,7 +2991,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="164" spans="1:8">
+    <row r="164" spans="1:7">
       <c r="A164" s="2" t="s">
         <v>175</v>
       </c>
@@ -3006,15 +3002,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:8">
+    <row r="165" spans="1:7">
       <c r="A165" s="2" t="s">
         <v>176</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7">
       <c r="A166" s="2" t="s">
         <v>177</v>
       </c>
@@ -3037,7 +3033,7 @@
         <v>0.26956018518518521</v>
       </c>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" spans="1:7">
       <c r="A167" s="2" t="s">
         <v>178</v>
       </c>
@@ -3048,7 +3044,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" spans="1:7">
       <c r="A168" s="2" t="s">
         <v>179</v>
       </c>
@@ -3059,7 +3055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" spans="1:7">
       <c r="A169" s="2" t="s">
         <v>180</v>
       </c>
@@ -3070,33 +3066,24 @@
         <v>0.14844907407407407</v>
       </c>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" spans="1:7">
       <c r="A170" s="2" t="s">
         <v>181</v>
       </c>
       <c r="B170" s="3">
-        <v>5.37037037037037E-3</v>
+        <v>4.6319444444444448E-2</v>
       </c>
       <c r="C170" s="3">
-        <v>2.5925925925925925E-2</v>
+        <v>0.14247685185185185</v>
       </c>
       <c r="D170" s="3">
-        <v>4.6319444444444448E-2</v>
+        <v>0.16750000000000001</v>
       </c>
       <c r="E170" s="3">
-        <v>0.14247685185185185</v>
-      </c>
-      <c r="F170" s="3">
-        <v>0.16750000000000001</v>
-      </c>
-      <c r="G170" s="3">
         <v>0.26238425925925923</v>
       </c>
-      <c r="H170" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="171" spans="1:8">
+    </row>
+    <row r="171" spans="1:7">
       <c r="A171" s="2" t="s">
         <v>182</v>
       </c>
@@ -3107,7 +3094,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" spans="1:7">
       <c r="A172" s="2" t="s">
         <v>183</v>
       </c>
@@ -3118,7 +3105,7 @@
         <v>0.10276620370370371</v>
       </c>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" spans="1:7">
       <c r="A173" s="2" t="s">
         <v>184</v>
       </c>
@@ -3129,7 +3116,7 @@
         <v>0.1575</v>
       </c>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" spans="1:7">
       <c r="A174" s="2" t="s">
         <v>185</v>
       </c>
@@ -3140,7 +3127,7 @@
         <v>0.17703703703703705</v>
       </c>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" spans="1:7">
       <c r="A175" s="2" t="s">
         <v>186</v>
       </c>
@@ -3151,7 +3138,7 @@
         <v>9.268518518518519E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:8">
+    <row r="176" spans="1:7">
       <c r="A176" s="2" t="s">
         <v>187</v>
       </c>
@@ -3175,7 +3162,7 @@
     </row>
     <row r="180" spans="1:3">
       <c r="C180" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="239" spans="1:1">

</xml_diff>

<commit_message>
on lab- redact video work and created make black segment deocde style + adds square in the corner
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F654748-8BDE-4DCF-B8EA-0C65F856E93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C226021E-B957-4E4D-9622-51CA8B3446C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="202">
   <si>
     <t>date</t>
   </si>
@@ -600,12 +611,6 @@
     <t>dead time</t>
   </si>
   <si>
-    <t>??</t>
-  </si>
-  <si>
-    <t>not a case</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 07:01:03</t>
   </si>
   <si>
@@ -631,6 +636,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>note a case</t>
+  </si>
+  <si>
+    <t>לא לחתוך</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1248,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:7">
       <c r="A17" s="2" t="s">
         <v>28</v>
       </c>
@@ -1260,7 +1271,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:7">
       <c r="A18" s="2" t="s">
         <v>29</v>
       </c>
@@ -1271,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:7">
       <c r="A19" s="2" t="s">
         <v>30</v>
       </c>
@@ -1282,7 +1293,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:7">
       <c r="A20" s="2" t="s">
         <v>31</v>
       </c>
@@ -1296,7 +1307,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
@@ -1307,7 +1318,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:7">
       <c r="A22" s="2" t="s">
         <v>33</v>
       </c>
@@ -1315,7 +1326,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:7">
       <c r="A23" s="2" t="s">
         <v>34</v>
       </c>
@@ -1326,7 +1337,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:7">
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
@@ -1337,7 +1348,7 @@
         <v>4.7546296296296295E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:7">
       <c r="A25" s="2" t="s">
         <v>36</v>
       </c>
@@ -1347,17 +1358,9 @@
       <c r="E25" s="3">
         <v>1.8576388888888889E-2</v>
       </c>
-      <c r="F25" s="3">
-        <v>3.1805555555555552E-2</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H25" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="2" t="s">
         <v>37</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>7.3530092592592591E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:7">
       <c r="A27" s="2" t="s">
         <v>38</v>
       </c>
@@ -1379,7 +1382,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:7">
       <c r="A28" s="2" t="s">
         <v>39</v>
       </c>
@@ -1390,7 +1393,7 @@
         <v>0.12725694444444444</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:7">
       <c r="A29" s="2" t="s">
         <v>40</v>
       </c>
@@ -1401,7 +1404,7 @@
         <v>0.25537037037037036</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:7">
       <c r="A30" s="2" t="s">
         <v>41</v>
       </c>
@@ -1412,7 +1415,7 @@
         <v>5.8252314814814812E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:7">
       <c r="A31" s="2" t="s">
         <v>42</v>
       </c>
@@ -1423,7 +1426,7 @@
         <v>8.5289351851851852E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:7">
       <c r="A32" s="2" t="s">
         <v>43</v>
       </c>
@@ -1434,7 +1437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:8">
       <c r="A33" s="2" t="s">
         <v>44</v>
       </c>
@@ -1445,7 +1448,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:8">
       <c r="A34" s="2" t="s">
         <v>45</v>
       </c>
@@ -1456,7 +1459,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
         <v>46</v>
       </c>
@@ -1467,7 +1470,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:8">
       <c r="A36" s="2" t="s">
         <v>47</v>
       </c>
@@ -1478,7 +1481,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
         <v>48</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:8">
       <c r="A38" s="2" t="s">
         <v>49</v>
       </c>
@@ -1500,7 +1503,7 @@
         <v>7.6284722222222226E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:8">
       <c r="A39" s="2" t="s">
         <v>50</v>
       </c>
@@ -1510,11 +1513,11 @@
       <c r="C39" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="H39" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="2" t="s">
         <v>51</v>
       </c>
@@ -1534,10 +1537,10 @@
         <v>0.22163194444444445</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" s="2" t="s">
         <v>52</v>
       </c>
@@ -1548,7 +1551,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:8">
       <c r="A42" s="2" t="s">
         <v>53</v>
       </c>
@@ -1559,7 +1562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:8">
       <c r="A43" s="2" t="s">
         <v>54</v>
       </c>
@@ -1570,7 +1573,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:8">
       <c r="A44" s="2" t="s">
         <v>55</v>
       </c>
@@ -1578,7 +1581,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:8">
       <c r="A45" s="2" t="s">
         <v>56</v>
       </c>
@@ -1589,7 +1592,7 @@
         <v>0.18371527777777777</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:8">
       <c r="A46" s="2" t="s">
         <v>57</v>
       </c>
@@ -1600,7 +1603,7 @@
         <v>0.12155092592592592</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:8">
       <c r="A47" s="2" t="s">
         <v>58</v>
       </c>
@@ -1611,7 +1614,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:8">
       <c r="A48" s="2" t="s">
         <v>59</v>
       </c>
@@ -1683,7 +1686,7 @@
         <v>0.19527777777777777</v>
       </c>
       <c r="H53" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -1702,7 +1705,7 @@
         <v>66</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C55" s="3">
         <v>9.6782407407407414E-2</v>
@@ -2029,12 +2032,8 @@
       <c r="C84" s="3">
         <v>0.12923611111111111</v>
       </c>
-      <c r="D84" s="3">
-        <v>0.15792824074074074</v>
-      </c>
-      <c r="E84" s="3">
-        <v>0.21453703703703703</v>
-      </c>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
       <c r="H84" t="s">
         <v>11</v>
       </c>
@@ -2082,11 +2081,8 @@
       <c r="C88" s="3">
         <v>5.6423611111111112E-2</v>
       </c>
-      <c r="D88" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="H88" t="s">
-        <v>11</v>
+      <c r="H88" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -2500,7 +2496,7 @@
         <v>129</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -2530,7 +2526,7 @@
         <v>132</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -2574,7 +2570,7 @@
         <v>9</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D125" s="3">
         <v>8.1180555555555561E-2</v>
@@ -2741,7 +2737,7 @@
         <v>9</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -2766,7 +2762,7 @@
         <v>151</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -2919,7 +2915,7 @@
         <v>166</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -2962,10 +2958,10 @@
         <v>171</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="161" spans="1:8">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7">
       <c r="A161" s="2" t="s">
         <v>172</v>
       </c>
@@ -2976,7 +2972,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8">
+    <row r="162" spans="1:7">
       <c r="A162" s="2" t="s">
         <v>173</v>
       </c>
@@ -2984,7 +2980,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="163" spans="1:8">
+    <row r="163" spans="1:7">
       <c r="A163" s="2" t="s">
         <v>174</v>
       </c>
@@ -2995,7 +2991,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="164" spans="1:8">
+    <row r="164" spans="1:7">
       <c r="A164" s="2" t="s">
         <v>175</v>
       </c>
@@ -3006,15 +3002,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:8">
+    <row r="165" spans="1:7">
       <c r="A165" s="2" t="s">
         <v>176</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7">
       <c r="A166" s="2" t="s">
         <v>177</v>
       </c>
@@ -3037,7 +3033,7 @@
         <v>0.26956018518518521</v>
       </c>
     </row>
-    <row r="167" spans="1:8">
+    <row r="167" spans="1:7">
       <c r="A167" s="2" t="s">
         <v>178</v>
       </c>
@@ -3048,7 +3044,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="168" spans="1:8">
+    <row r="168" spans="1:7">
       <c r="A168" s="2" t="s">
         <v>179</v>
       </c>
@@ -3059,7 +3055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="1:8">
+    <row r="169" spans="1:7">
       <c r="A169" s="2" t="s">
         <v>180</v>
       </c>
@@ -3070,33 +3066,24 @@
         <v>0.14844907407407407</v>
       </c>
     </row>
-    <row r="170" spans="1:8">
+    <row r="170" spans="1:7">
       <c r="A170" s="2" t="s">
         <v>181</v>
       </c>
       <c r="B170" s="3">
-        <v>5.37037037037037E-3</v>
+        <v>4.6319444444444448E-2</v>
       </c>
       <c r="C170" s="3">
-        <v>2.5925925925925925E-2</v>
+        <v>0.14247685185185185</v>
       </c>
       <c r="D170" s="3">
-        <v>4.6319444444444448E-2</v>
+        <v>0.16750000000000001</v>
       </c>
       <c r="E170" s="3">
-        <v>0.14247685185185185</v>
-      </c>
-      <c r="F170" s="3">
-        <v>0.16750000000000001</v>
-      </c>
-      <c r="G170" s="3">
         <v>0.26238425925925923</v>
       </c>
-      <c r="H170" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="171" spans="1:8">
+    </row>
+    <row r="171" spans="1:7">
       <c r="A171" s="2" t="s">
         <v>182</v>
       </c>
@@ -3107,7 +3094,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="172" spans="1:8">
+    <row r="172" spans="1:7">
       <c r="A172" s="2" t="s">
         <v>183</v>
       </c>
@@ -3118,7 +3105,7 @@
         <v>0.10276620370370371</v>
       </c>
     </row>
-    <row r="173" spans="1:8">
+    <row r="173" spans="1:7">
       <c r="A173" s="2" t="s">
         <v>184</v>
       </c>
@@ -3129,7 +3116,7 @@
         <v>0.1575</v>
       </c>
     </row>
-    <row r="174" spans="1:8">
+    <row r="174" spans="1:7">
       <c r="A174" s="2" t="s">
         <v>185</v>
       </c>
@@ -3140,7 +3127,7 @@
         <v>0.17703703703703705</v>
       </c>
     </row>
-    <row r="175" spans="1:8">
+    <row r="175" spans="1:7">
       <c r="A175" s="2" t="s">
         <v>186</v>
       </c>
@@ -3151,7 +3138,7 @@
         <v>9.268518518518519E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:8">
+    <row r="176" spans="1:7">
       <c r="A176" s="2" t="s">
         <v>187</v>
       </c>
@@ -3175,7 +3162,7 @@
     </row>
     <row r="180" spans="1:3">
       <c r="C180" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="239" spans="1:1">

</xml_diff>

<commit_message>
add cols to db and make sure batch redact is updates it
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Python\ScalpelLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA199D4A-A65B-42BB-8493-DE1B8EC648A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C05E792-E7A6-40ED-A18F-6FE1F836C006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -795,18 +795,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H243"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="45.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17.69921875" style="2" customWidth="1"/>
     <col min="6" max="6" width="16.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.8984375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>129</v>
       </c>

</xml_diff>

<commit_message>
Add database columns and keep batch redaction in sync
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Room_8_Data\Scalpel_Raz\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Python\ScalpelLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA199D4A-A65B-42BB-8493-DE1B8EC648A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C05E792-E7A6-40ED-A18F-6FE1F836C006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -795,18 +795,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H243"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="45.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.09765625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.75" style="2" customWidth="1"/>
+    <col min="5" max="5" width="17.69921875" style="2" customWidth="1"/>
     <col min="6" max="6" width="16.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.8984375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>129</v>
       </c>

</xml_diff>